<commit_message>
docs: bo sung so do quan he CSDL ERD kem mui ten chi ro moi lien ket va bang anh xa khoa ngoai
</commit_message>
<xml_diff>
--- a/khởi động/CineMax_AI_ChucNang_Va_Database_Giong_Mau.xlsx
+++ b/khởi động/CineMax_AI_ChucNang_Va_Database_Giong_Mau.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CHỨC NĂNG" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DATABASE (11 BẢNG)" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="THÀNH VIÊN DỰ ÁN" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SƠ ĐỒ LIÊN KẾT ERD" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="16">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -116,6 +117,18 @@
       <color rgb="001E3A8A"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001E3A8A"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <b val="1"/>
+      <color rgb="000284C7"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="9">
     <fill>
@@ -167,7 +180,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -203,11 +216,55 @@
         <color rgb="001E3A8A"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -329,6 +386,21 @@
     <xf numFmtId="0" fontId="15" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -403,6 +475,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10477500" cy="6953250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1775,13 +1877,13 @@
           <t>BẢNG DỮ LIỆU: USERS</t>
         </is>
       </c>
-      <c r="B6" s="29" t="n"/>
-      <c r="C6" s="29" t="n"/>
-      <c r="D6" s="29" t="n"/>
-      <c r="E6" s="29" t="n"/>
-      <c r="F6" s="29" t="n"/>
-      <c r="G6" s="29" t="n"/>
-      <c r="H6" s="29" t="n"/>
+      <c r="B6" s="45" t="n"/>
+      <c r="C6" s="45" t="n"/>
+      <c r="D6" s="45" t="n"/>
+      <c r="E6" s="45" t="n"/>
+      <c r="F6" s="45" t="n"/>
+      <c r="G6" s="45" t="n"/>
+      <c r="H6" s="46" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="30" t="inlineStr">
@@ -2161,13 +2263,13 @@
           <t>BẢNG DỮ LIỆU: CINEMAS</t>
         </is>
       </c>
-      <c r="B18" s="29" t="n"/>
-      <c r="C18" s="29" t="n"/>
-      <c r="D18" s="29" t="n"/>
-      <c r="E18" s="29" t="n"/>
-      <c r="F18" s="29" t="n"/>
-      <c r="G18" s="29" t="n"/>
-      <c r="H18" s="29" t="n"/>
+      <c r="B18" s="45" t="n"/>
+      <c r="C18" s="45" t="n"/>
+      <c r="D18" s="45" t="n"/>
+      <c r="E18" s="45" t="n"/>
+      <c r="F18" s="45" t="n"/>
+      <c r="G18" s="45" t="n"/>
+      <c r="H18" s="46" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="30" t="inlineStr">
@@ -2403,13 +2505,13 @@
           <t>BẢNG DỮ LIỆU: ROOMS</t>
         </is>
       </c>
-      <c r="B26" s="29" t="n"/>
-      <c r="C26" s="29" t="n"/>
-      <c r="D26" s="29" t="n"/>
-      <c r="E26" s="29" t="n"/>
-      <c r="F26" s="29" t="n"/>
-      <c r="G26" s="29" t="n"/>
-      <c r="H26" s="29" t="n"/>
+      <c r="B26" s="45" t="n"/>
+      <c r="C26" s="45" t="n"/>
+      <c r="D26" s="45" t="n"/>
+      <c r="E26" s="45" t="n"/>
+      <c r="F26" s="45" t="n"/>
+      <c r="G26" s="45" t="n"/>
+      <c r="H26" s="46" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="30" t="inlineStr">
@@ -2649,13 +2751,13 @@
           <t>BẢNG DỮ LIỆU: MOVIES</t>
         </is>
       </c>
-      <c r="B34" s="29" t="n"/>
-      <c r="C34" s="29" t="n"/>
-      <c r="D34" s="29" t="n"/>
-      <c r="E34" s="29" t="n"/>
-      <c r="F34" s="29" t="n"/>
-      <c r="G34" s="29" t="n"/>
-      <c r="H34" s="29" t="n"/>
+      <c r="B34" s="45" t="n"/>
+      <c r="C34" s="45" t="n"/>
+      <c r="D34" s="45" t="n"/>
+      <c r="E34" s="45" t="n"/>
+      <c r="F34" s="45" t="n"/>
+      <c r="G34" s="45" t="n"/>
+      <c r="H34" s="46" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="30" t="inlineStr">
@@ -3111,13 +3213,13 @@
           <t>BẢNG DỮ LIỆU: SHOWTIMES</t>
         </is>
       </c>
-      <c r="B48" s="29" t="n"/>
-      <c r="C48" s="29" t="n"/>
-      <c r="D48" s="29" t="n"/>
-      <c r="E48" s="29" t="n"/>
-      <c r="F48" s="29" t="n"/>
-      <c r="G48" s="29" t="n"/>
-      <c r="H48" s="29" t="n"/>
+      <c r="B48" s="45" t="n"/>
+      <c r="C48" s="45" t="n"/>
+      <c r="D48" s="45" t="n"/>
+      <c r="E48" s="45" t="n"/>
+      <c r="F48" s="45" t="n"/>
+      <c r="G48" s="45" t="n"/>
+      <c r="H48" s="46" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="30" t="inlineStr">
@@ -3501,13 +3603,13 @@
           <t>BẢNG DỮ LIỆU: SEAT_LAYOUTS</t>
         </is>
       </c>
-      <c r="B60" s="29" t="n"/>
-      <c r="C60" s="29" t="n"/>
-      <c r="D60" s="29" t="n"/>
-      <c r="E60" s="29" t="n"/>
-      <c r="F60" s="29" t="n"/>
-      <c r="G60" s="29" t="n"/>
-      <c r="H60" s="29" t="n"/>
+      <c r="B60" s="45" t="n"/>
+      <c r="C60" s="45" t="n"/>
+      <c r="D60" s="45" t="n"/>
+      <c r="E60" s="45" t="n"/>
+      <c r="F60" s="45" t="n"/>
+      <c r="G60" s="45" t="n"/>
+      <c r="H60" s="46" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="30" t="inlineStr">
@@ -3701,13 +3803,13 @@
           <t>BẢNG DỮ LIỆU: SEAT_HOLDS</t>
         </is>
       </c>
-      <c r="B67" s="29" t="n"/>
-      <c r="C67" s="29" t="n"/>
-      <c r="D67" s="29" t="n"/>
-      <c r="E67" s="29" t="n"/>
-      <c r="F67" s="29" t="n"/>
-      <c r="G67" s="29" t="n"/>
-      <c r="H67" s="29" t="n"/>
+      <c r="B67" s="45" t="n"/>
+      <c r="C67" s="45" t="n"/>
+      <c r="D67" s="45" t="n"/>
+      <c r="E67" s="45" t="n"/>
+      <c r="F67" s="45" t="n"/>
+      <c r="G67" s="45" t="n"/>
+      <c r="H67" s="46" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="34" t="inlineStr">
@@ -3939,13 +4041,13 @@
           <t>BẢNG DỮ LIỆU: BOOKINGS</t>
         </is>
       </c>
-      <c r="B75" s="29" t="n"/>
-      <c r="C75" s="29" t="n"/>
-      <c r="D75" s="29" t="n"/>
-      <c r="E75" s="29" t="n"/>
-      <c r="F75" s="29" t="n"/>
-      <c r="G75" s="29" t="n"/>
-      <c r="H75" s="29" t="n"/>
+      <c r="B75" s="45" t="n"/>
+      <c r="C75" s="45" t="n"/>
+      <c r="D75" s="45" t="n"/>
+      <c r="E75" s="45" t="n"/>
+      <c r="F75" s="45" t="n"/>
+      <c r="G75" s="45" t="n"/>
+      <c r="H75" s="46" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="34" t="inlineStr">
@@ -4473,13 +4575,13 @@
           <t>BẢNG DỮ LIỆU: TICKETS</t>
         </is>
       </c>
-      <c r="B91" s="29" t="n"/>
-      <c r="C91" s="29" t="n"/>
-      <c r="D91" s="29" t="n"/>
-      <c r="E91" s="29" t="n"/>
-      <c r="F91" s="29" t="n"/>
-      <c r="G91" s="29" t="n"/>
-      <c r="H91" s="29" t="n"/>
+      <c r="B91" s="45" t="n"/>
+      <c r="C91" s="45" t="n"/>
+      <c r="D91" s="45" t="n"/>
+      <c r="E91" s="45" t="n"/>
+      <c r="F91" s="45" t="n"/>
+      <c r="G91" s="45" t="n"/>
+      <c r="H91" s="46" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="34" t="inlineStr">
@@ -4749,13 +4851,13 @@
           <t>BẢNG DỮ LIỆU: VOUCHERS</t>
         </is>
       </c>
-      <c r="B100" s="29" t="n"/>
-      <c r="C100" s="29" t="n"/>
-      <c r="D100" s="29" t="n"/>
-      <c r="E100" s="29" t="n"/>
-      <c r="F100" s="29" t="n"/>
-      <c r="G100" s="29" t="n"/>
-      <c r="H100" s="29" t="n"/>
+      <c r="B100" s="45" t="n"/>
+      <c r="C100" s="45" t="n"/>
+      <c r="D100" s="45" t="n"/>
+      <c r="E100" s="45" t="n"/>
+      <c r="F100" s="45" t="n"/>
+      <c r="G100" s="45" t="n"/>
+      <c r="H100" s="46" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="30" t="inlineStr">
@@ -5157,13 +5259,13 @@
           <t>BẢNG DỮ LIỆU: REVIEWS</t>
         </is>
       </c>
-      <c r="B113" s="29" t="n"/>
-      <c r="C113" s="29" t="n"/>
-      <c r="D113" s="29" t="n"/>
-      <c r="E113" s="29" t="n"/>
-      <c r="F113" s="29" t="n"/>
-      <c r="G113" s="29" t="n"/>
-      <c r="H113" s="29" t="n"/>
+      <c r="B113" s="45" t="n"/>
+      <c r="C113" s="45" t="n"/>
+      <c r="D113" s="45" t="n"/>
+      <c r="E113" s="45" t="n"/>
+      <c r="F113" s="45" t="n"/>
+      <c r="G113" s="45" t="n"/>
+      <c r="H113" s="46" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="34" t="inlineStr">
@@ -5673,4 +5775,645 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:I59"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="65" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="A2" s="47" t="inlineStr">
+        <is>
+          <t>SƠ ĐỒ QUAN HỆ &amp; BẢNG ÁNH XẠ MỐI LIÊN KẾT CƠ SỞ DỮ LIỆU (ERD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="27" t="inlineStr">
+        <is>
+          <t>Đặc tả trực quan 11 bảng dữ liệu, khóa chính (PK), khóa ngoại (FK), mũi tên liên kết và bản số (Cardinality 1:N, 1:1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="47" t="inlineStr">
+        <is>
+          <t>BẢNG QUAN HỆ &amp; RÀNG BUỘC TOÀN VẸN KHÓA NGOẠI (FOREIGN KEY MAPPING MATRIX)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="27" t="inlineStr">
+        <is>
+          <t>Chi tiết các đường liên kết giữa các thực thể, bản số và quy tắc toàn vẹn dữ liệu</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Bảng Nguồn (Parent)</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>Khóa Chính (PK)</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Bản Số</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Mũi Tên Liên Kết (Relationship)</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>Bảng Đích (Child)</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>Khóa Ngoại (FK)</t>
+        </is>
+      </c>
+      <c r="H47" s="5" t="inlineStr">
+        <is>
+          <t>Ràng Buộc (Cascade/Restrict)</t>
+        </is>
+      </c>
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t>Ý Nghĩa Nghiệp Vụ Cốt Lõi</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="B48" s="41" t="inlineStr">
+        <is>
+          <t>cinemas</t>
+        </is>
+      </c>
+      <c r="C48" s="40" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="D48" s="41" t="inlineStr">
+        <is>
+          <t>1 : N</t>
+        </is>
+      </c>
+      <c r="E48" s="48" t="inlineStr">
+        <is>
+          <t>────────(1 : N)────────►</t>
+        </is>
+      </c>
+      <c r="F48" s="41" t="inlineStr">
+        <is>
+          <t>rooms</t>
+        </is>
+      </c>
+      <c r="G48" s="38" t="inlineStr">
+        <is>
+          <t>cinema_id</t>
+        </is>
+      </c>
+      <c r="H48" s="41" t="inlineStr">
+        <is>
+          <t>CASCADE</t>
+        </is>
+      </c>
+      <c r="I48" s="49" t="inlineStr">
+        <is>
+          <t>Một cụm rạp quản lý nhiều phòng chiếu (Phòng Standard, IMAX Laser, ScreenX). Xóa rạp thì xóa phòng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="43" t="n">
+        <v>2</v>
+      </c>
+      <c r="B49" s="43" t="inlineStr">
+        <is>
+          <t>cinemas</t>
+        </is>
+      </c>
+      <c r="C49" s="32" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="D49" s="43" t="inlineStr">
+        <is>
+          <t>1 : N</t>
+        </is>
+      </c>
+      <c r="E49" s="50" t="inlineStr">
+        <is>
+          <t>────────(1 : N)────────►</t>
+        </is>
+      </c>
+      <c r="F49" s="43" t="inlineStr">
+        <is>
+          <t>showtimes</t>
+        </is>
+      </c>
+      <c r="G49" s="39" t="inlineStr">
+        <is>
+          <t>cinema_id</t>
+        </is>
+      </c>
+      <c r="H49" s="43" t="inlineStr">
+        <is>
+          <t>RESTRICT</t>
+        </is>
+      </c>
+      <c r="I49" s="51" t="inlineStr">
+        <is>
+          <t>Một cụm rạp tổ chức nhiều suất chiếu. Không được xóa rạp nếu đang có suất chiếu tương lai.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="41" t="n">
+        <v>3</v>
+      </c>
+      <c r="B50" s="41" t="inlineStr">
+        <is>
+          <t>rooms</t>
+        </is>
+      </c>
+      <c r="C50" s="40" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="D50" s="41" t="inlineStr">
+        <is>
+          <t>1 : N</t>
+        </is>
+      </c>
+      <c r="E50" s="48" t="inlineStr">
+        <is>
+          <t>────────(1 : N)────────►</t>
+        </is>
+      </c>
+      <c r="F50" s="41" t="inlineStr">
+        <is>
+          <t>seat_layouts</t>
+        </is>
+      </c>
+      <c r="G50" s="38" t="inlineStr">
+        <is>
+          <t>room_id</t>
+        </is>
+      </c>
+      <c r="H50" s="41" t="inlineStr">
+        <is>
+          <t>CASCADE</t>
+        </is>
+      </c>
+      <c r="I50" s="49" t="inlineStr">
+        <is>
+          <t>Một phòng chiếu sở hữu cấu hình sơ đồ 102 ghế cố định (A1-H12, K1-K6).</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="B51" s="43" t="inlineStr">
+        <is>
+          <t>rooms</t>
+        </is>
+      </c>
+      <c r="C51" s="32" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="D51" s="43" t="inlineStr">
+        <is>
+          <t>1 : N</t>
+        </is>
+      </c>
+      <c r="E51" s="50" t="inlineStr">
+        <is>
+          <t>────────(1 : N)────────►</t>
+        </is>
+      </c>
+      <c r="F51" s="43" t="inlineStr">
+        <is>
+          <t>showtimes</t>
+        </is>
+      </c>
+      <c r="G51" s="39" t="inlineStr">
+        <is>
+          <t>room_id</t>
+        </is>
+      </c>
+      <c r="H51" s="43" t="inlineStr">
+        <is>
+          <t>RESTRICT</t>
+        </is>
+      </c>
+      <c r="I51" s="51" t="inlineStr">
+        <is>
+          <t>Một phòng chiếu tổ chức nhiều suất chiếu. Showtime Collision Engine kiểm tra không trùng giờ trên cùng 1 room_id.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="41" t="n">
+        <v>5</v>
+      </c>
+      <c r="B52" s="41" t="inlineStr">
+        <is>
+          <t>movies</t>
+        </is>
+      </c>
+      <c r="C52" s="40" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="D52" s="41" t="inlineStr">
+        <is>
+          <t>1 : N</t>
+        </is>
+      </c>
+      <c r="E52" s="48" t="inlineStr">
+        <is>
+          <t>────────(1 : N)────────►</t>
+        </is>
+      </c>
+      <c r="F52" s="41" t="inlineStr">
+        <is>
+          <t>showtimes</t>
+        </is>
+      </c>
+      <c r="G52" s="38" t="inlineStr">
+        <is>
+          <t>movie_id</t>
+        </is>
+      </c>
+      <c r="H52" s="41" t="inlineStr">
+        <is>
+          <t>RESTRICT</t>
+        </is>
+      </c>
+      <c r="I52" s="49" t="inlineStr">
+        <is>
+          <t>Một bộ phim được xếp lịch chiếu tại nhiều khung giờ và rạp khác nhau. Dùng duration_minutes để tính thời lượng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="43" t="n">
+        <v>6</v>
+      </c>
+      <c r="B53" s="43" t="inlineStr">
+        <is>
+          <t>movies</t>
+        </is>
+      </c>
+      <c r="C53" s="32" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="D53" s="43" t="inlineStr">
+        <is>
+          <t>1 : N</t>
+        </is>
+      </c>
+      <c r="E53" s="50" t="inlineStr">
+        <is>
+          <t>────────(1 : N)────────►</t>
+        </is>
+      </c>
+      <c r="F53" s="43" t="inlineStr">
+        <is>
+          <t>reviews</t>
+        </is>
+      </c>
+      <c r="G53" s="39" t="inlineStr">
+        <is>
+          <t>movie_id</t>
+        </is>
+      </c>
+      <c r="H53" s="43" t="inlineStr">
+        <is>
+          <t>CASCADE</t>
+        </is>
+      </c>
+      <c r="I53" s="51" t="inlineStr">
+        <is>
+          <t>Một bộ phim nhận được nhiều nhận xét đánh giá từ khán giả. Xóa phim sẽ xóa các đánh giá liên quan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="41" t="n">
+        <v>7</v>
+      </c>
+      <c r="B54" s="41" t="inlineStr">
+        <is>
+          <t>showtimes</t>
+        </is>
+      </c>
+      <c r="C54" s="40" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="D54" s="41" t="inlineStr">
+        <is>
+          <t>1 : N</t>
+        </is>
+      </c>
+      <c r="E54" s="48" t="inlineStr">
+        <is>
+          <t>────────(1 : N)────────►</t>
+        </is>
+      </c>
+      <c r="F54" s="41" t="inlineStr">
+        <is>
+          <t>seat_holds</t>
+        </is>
+      </c>
+      <c r="G54" s="38" t="inlineStr">
+        <is>
+          <t>showtime_id</t>
+        </is>
+      </c>
+      <c r="H54" s="41" t="inlineStr">
+        <is>
+          <t>CASCADE</t>
+        </is>
+      </c>
+      <c r="I54" s="49" t="inlineStr">
+        <is>
+          <t>Một suất chiếu có nhiều phiên giữ ghế tạm thời. Redis Key: cinemax:{showtimeId}:hold:{holdId} với TTL 300s.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="43" t="n">
+        <v>8</v>
+      </c>
+      <c r="B55" s="43" t="inlineStr">
+        <is>
+          <t>showtimes</t>
+        </is>
+      </c>
+      <c r="C55" s="32" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="D55" s="43" t="inlineStr">
+        <is>
+          <t>1 : N</t>
+        </is>
+      </c>
+      <c r="E55" s="50" t="inlineStr">
+        <is>
+          <t>────────(1 : N)────────►</t>
+        </is>
+      </c>
+      <c r="F55" s="43" t="inlineStr">
+        <is>
+          <t>bookings</t>
+        </is>
+      </c>
+      <c r="G55" s="39" t="inlineStr">
+        <is>
+          <t>showtime_id</t>
+        </is>
+      </c>
+      <c r="H55" s="43" t="inlineStr">
+        <is>
+          <t>RESTRICT</t>
+        </is>
+      </c>
+      <c r="I55" s="51" t="inlineStr">
+        <is>
+          <t>Một suất chiếu có nhiều đơn đặt vé đã thanh toán thành công. Không thể xóa suất chiếu nếu đã bán vé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="41" t="n">
+        <v>9</v>
+      </c>
+      <c r="B56" s="41" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="C56" s="40" t="inlineStr">
+        <is>
+          <t>id / phone</t>
+        </is>
+      </c>
+      <c r="D56" s="41" t="inlineStr">
+        <is>
+          <t>1 : N</t>
+        </is>
+      </c>
+      <c r="E56" s="48" t="inlineStr">
+        <is>
+          <t>────────(1 : N)────────►</t>
+        </is>
+      </c>
+      <c r="F56" s="41" t="inlineStr">
+        <is>
+          <t>bookings</t>
+        </is>
+      </c>
+      <c r="G56" s="38" t="inlineStr">
+        <is>
+          <t>customer_phone</t>
+        </is>
+      </c>
+      <c r="H56" s="41" t="inlineStr">
+        <is>
+          <t>SET NULL</t>
+        </is>
+      </c>
+      <c r="I56" s="49" t="inlineStr">
+        <is>
+          <t>Một tài khoản người dùng / số điện thoại thực hiện nhiều đơn đặt vé. Dùng để xem lịch sử vé tại /dashboard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="43" t="n">
+        <v>10</v>
+      </c>
+      <c r="B57" s="43" t="inlineStr">
+        <is>
+          <t>vouchers</t>
+        </is>
+      </c>
+      <c r="C57" s="32" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="D57" s="43" t="inlineStr">
+        <is>
+          <t>1 : N</t>
+        </is>
+      </c>
+      <c r="E57" s="50" t="inlineStr">
+        <is>
+          <t>────────(1 : N)────────►</t>
+        </is>
+      </c>
+      <c r="F57" s="43" t="inlineStr">
+        <is>
+          <t>bookings</t>
+        </is>
+      </c>
+      <c r="G57" s="39" t="inlineStr">
+        <is>
+          <t>voucher_code</t>
+        </is>
+      </c>
+      <c r="H57" s="43" t="inlineStr">
+        <is>
+          <t>SET NULL</t>
+        </is>
+      </c>
+      <c r="I57" s="51" t="inlineStr">
+        <is>
+          <t>Một mã khuyến mãi có thể được áp dụng cho nhiều đơn vé khác nhau cho đến khi hết hạn mức usage_limit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="41" t="n">
+        <v>11</v>
+      </c>
+      <c r="B58" s="41" t="inlineStr">
+        <is>
+          <t>bookings</t>
+        </is>
+      </c>
+      <c r="C58" s="40" t="inlineStr">
+        <is>
+          <t>booking_id</t>
+        </is>
+      </c>
+      <c r="D58" s="41" t="inlineStr">
+        <is>
+          <t>1 : 1</t>
+        </is>
+      </c>
+      <c r="E58" s="48" t="inlineStr">
+        <is>
+          <t>────────(1 : 1)────────►</t>
+        </is>
+      </c>
+      <c r="F58" s="41" t="inlineStr">
+        <is>
+          <t>tickets</t>
+        </is>
+      </c>
+      <c r="G58" s="38" t="inlineStr">
+        <is>
+          <t>booking_id</t>
+        </is>
+      </c>
+      <c r="H58" s="41" t="inlineStr">
+        <is>
+          <t>CASCADE</t>
+        </is>
+      </c>
+      <c r="I58" s="49" t="inlineStr">
+        <is>
+          <t>Quan hệ 1-1 CHẶT CHẼ: Mỗi đơn đặt vé phát hành DUY NHẤT 1 vé điện tử chứa chuỗi mã QR ký số HMAC-SHA256.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="43" t="n">
+        <v>12</v>
+      </c>
+      <c r="B59" s="43" t="inlineStr">
+        <is>
+          <t>bookings</t>
+        </is>
+      </c>
+      <c r="C59" s="32" t="inlineStr">
+        <is>
+          <t>booking_id</t>
+        </is>
+      </c>
+      <c r="D59" s="43" t="inlineStr">
+        <is>
+          <t>1 : 1</t>
+        </is>
+      </c>
+      <c r="E59" s="50" t="inlineStr">
+        <is>
+          <t>────────(1 : 1)────────►</t>
+        </is>
+      </c>
+      <c r="F59" s="43" t="inlineStr">
+        <is>
+          <t>reviews</t>
+        </is>
+      </c>
+      <c r="G59" s="39" t="inlineStr">
+        <is>
+          <t>booking_id</t>
+        </is>
+      </c>
+      <c r="H59" s="43" t="inlineStr">
+        <is>
+          <t>SET NULL</t>
+        </is>
+      </c>
+      <c r="I59" s="51" t="inlineStr">
+        <is>
+          <t>Quan hệ 1-1 BẢO MẬT: Mỗi đơn vé chỉ được đánh giá phim 1 lần duy nhất (Verified Review chống đánh giá ảo).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>